<commit_message>
Resultados - PR (Etapa 1)
</commit_message>
<xml_diff>
--- a/resultados/abatia/erros_varredura.xlsx
+++ b/resultados/abatia/erros_varredura.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F388"/>
+  <dimension ref="A1:F451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11284,6 +11284,1770 @@
         </is>
       </c>
     </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=00CDF12EB8D3827634D79C05009B0FE1?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=AGOSTO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D389" t="n">
+        <v>0</v>
+      </c>
+      <c r="E389" t="n">
+        <v>6</v>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>2026-07-31 22:57:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=19E48E5593B51B8203CFF5A29E206288?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=AGOSTO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D390" t="n">
+        <v>0</v>
+      </c>
+      <c r="E390" t="n">
+        <v>6</v>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:01:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=1DB0E756E1C061D09AAF974F1B434815?d-5470-p=4&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=AGOSTO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D391" t="n">
+        <v>0</v>
+      </c>
+      <c r="E391" t="n">
+        <v>6</v>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:02:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=DDCE7B8A1B7D2EEB88A1D472B3B244A0?d-5470-p=4&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=SETEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D392" t="n">
+        <v>0</v>
+      </c>
+      <c r="E392" t="n">
+        <v>6</v>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:10:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=A1B48967BAF8E1A635EEFDA5BA9E6EDE?d-5470-p=4&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=SETEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D393" t="n">
+        <v>0</v>
+      </c>
+      <c r="E393" t="n">
+        <v>6</v>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:17:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=2B708D2A1E30C8C83D8A666ABB166ED6?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>0</v>
+      </c>
+      <c r="E394" t="n">
+        <v>6</v>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:20:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=3D5D88D14E91F9444A6F30EE76BE5162?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D395" t="n">
+        <v>0</v>
+      </c>
+      <c r="E395" t="n">
+        <v>6</v>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:24:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=031CE6644B7B7A86C78BCD00EC265964?d-5470-p=4&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D396" t="n">
+        <v>0</v>
+      </c>
+      <c r="E396" t="n">
+        <v>6</v>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:25:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=A1EEB9106F51B21BE7BFC2F64846356D?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D397" t="n">
+        <v>0</v>
+      </c>
+      <c r="E397" t="n">
+        <v>6</v>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:27:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=6FBC8CA7C2924E7F7B566C80341B27A5?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D398" t="n">
+        <v>0</v>
+      </c>
+      <c r="E398" t="n">
+        <v>6</v>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:29:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=11C4EF694DFF3D359586E6EE0B46155E?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D399" t="n">
+        <v>0</v>
+      </c>
+      <c r="E399" t="n">
+        <v>6</v>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:30:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=5748551C0F41482D845FC54E70424F07?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D400" t="n">
+        <v>0</v>
+      </c>
+      <c r="E400" t="n">
+        <v>6</v>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:33:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=6C8330313B889778B1CED8FF1AF4F1B6?d-5470-p=3&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D401" t="n">
+        <v>0</v>
+      </c>
+      <c r="E401" t="n">
+        <v>6</v>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:34:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=2C891E4E5E8CFAAC6F35535328C8597E?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>0</v>
+      </c>
+      <c r="E402" t="n">
+        <v>6</v>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:34:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=4B68EFAD66F280E3B7F72BA7492696E5?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D403" t="n">
+        <v>0</v>
+      </c>
+      <c r="E403" t="n">
+        <v>6</v>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:38:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=914D4CD203ED6AAC8189DABAD1CCC7E1?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D404" t="n">
+        <v>0</v>
+      </c>
+      <c r="E404" t="n">
+        <v>6</v>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:39:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=1F51CA6EF2BEEDEB953F3B8C8AFBC8AE?d-5470-p=4&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>0</v>
+      </c>
+      <c r="E405" t="n">
+        <v>6</v>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:40:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=FF14E97F6367793E64A77A1DCAC2A723?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D406" t="n">
+        <v>0</v>
+      </c>
+      <c r="E406" t="n">
+        <v>6</v>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:41:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=DD04C372CBF4B7BA194C4B02E7B2417F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=2&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>TIMEOUT_OU_CONEXAO</t>
+        </is>
+      </c>
+      <c r="D407" t="n">
+        <v>0</v>
+      </c>
+      <c r="E407" t="n">
+        <v>6</v>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:43:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=DD04C372CBF4B7BA194C4B02E7B2417F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=2&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D408" t="n">
+        <v>0</v>
+      </c>
+      <c r="E408" t="n">
+        <v>6</v>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:43:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=DD04C372CBF4B7BA194C4B02E7B2417F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=5&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>TIMEOUT_OU_CONEXAO</t>
+        </is>
+      </c>
+      <c r="D409" t="n">
+        <v>0</v>
+      </c>
+      <c r="E409" t="n">
+        <v>6</v>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:43:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=DD04C372CBF4B7BA194C4B02E7B2417F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=5&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>0</v>
+      </c>
+      <c r="E410" t="n">
+        <v>6</v>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:43:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=DD04C372CBF4B7BA194C4B02E7B2417F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=6&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>TIMEOUT_OU_CONEXAO</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>0</v>
+      </c>
+      <c r="E411" t="n">
+        <v>6</v>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:43:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=DD04C372CBF4B7BA194C4B02E7B2417F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=6&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D412" t="n">
+        <v>0</v>
+      </c>
+      <c r="E412" t="n">
+        <v>6</v>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:43:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=DD04C372CBF4B7BA194C4B02E7B2417F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>TIMEOUT_OU_CONEXAO</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>0</v>
+      </c>
+      <c r="E413" t="n">
+        <v>6</v>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:43:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=DD04C372CBF4B7BA194C4B02E7B2417F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>0</v>
+      </c>
+      <c r="E414" t="n">
+        <v>6</v>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:43:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=82A7F1F8C0C6EFDAC7CC73B35084CD60?d-5470-p=3&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>0</v>
+      </c>
+      <c r="E415" t="n">
+        <v>6</v>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:44:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=75C9657509AD83D7ACED45763BE2A976?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=1&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>TIMEOUT_OU_CONEXAO</t>
+        </is>
+      </c>
+      <c r="D416" t="n">
+        <v>0</v>
+      </c>
+      <c r="E416" t="n">
+        <v>6</v>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:45:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=75C9657509AD83D7ACED45763BE2A976?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=1&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D417" t="n">
+        <v>0</v>
+      </c>
+      <c r="E417" t="n">
+        <v>6</v>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:45:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=75C9657509AD83D7ACED45763BE2A976?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=2&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>TIMEOUT_OU_CONEXAO</t>
+        </is>
+      </c>
+      <c r="D418" t="n">
+        <v>0</v>
+      </c>
+      <c r="E418" t="n">
+        <v>6</v>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:45:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=75C9657509AD83D7ACED45763BE2A976?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=2&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D419" t="n">
+        <v>0</v>
+      </c>
+      <c r="E419" t="n">
+        <v>6</v>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:45:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=75C9657509AD83D7ACED45763BE2A976?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D420" t="n">
+        <v>0</v>
+      </c>
+      <c r="E420" t="n">
+        <v>6</v>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:46:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=75C9657509AD83D7ACED45763BE2A976?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=10&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>TIMEOUT_OU_CONEXAO</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>0</v>
+      </c>
+      <c r="E421" t="n">
+        <v>6</v>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:46:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=75C9657509AD83D7ACED45763BE2A976?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=10&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D422" t="n">
+        <v>0</v>
+      </c>
+      <c r="E422" t="n">
+        <v>6</v>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:46:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=5B499ADAF587097CDE08F70729538AA6?d-5470-p=4&amp;formulario.exercicio=2020&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>TIMEOUT_OU_CONEXAO</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>0</v>
+      </c>
+      <c r="E423" t="n">
+        <v>6</v>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:47:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=5B499ADAF587097CDE08F70729538AA6?d-5470-p=4&amp;formulario.exercicio=2020&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>0</v>
+      </c>
+      <c r="E424" t="n">
+        <v>6</v>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:47:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=5B499ADAF587097CDE08F70729538AA6?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>0</v>
+      </c>
+      <c r="E425" t="n">
+        <v>6</v>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:47:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=83C9119E917F1546C67CDF011D51654D?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>0</v>
+      </c>
+      <c r="E426" t="n">
+        <v>6</v>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:48:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=878E5C91B0B20A2CF304DBC6082946EB?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>0</v>
+      </c>
+      <c r="E427" t="n">
+        <v>6</v>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:50:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=95801FFDA2EADE807BFF13578096A695?d-5470-p=3&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=NOVEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>0</v>
+      </c>
+      <c r="E428" t="n">
+        <v>6</v>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:51:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=354578055FFE8964BEBE7E7A0CAA447D?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=DEZEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>0</v>
+      </c>
+      <c r="E429" t="n">
+        <v>6</v>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:52:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=9908FD8AA7E2A23E3F4790C841C88588?d-5470-p=3&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=DEZEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>0</v>
+      </c>
+      <c r="E430" t="n">
+        <v>6</v>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:53:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=C6B40012BEA5C5A631F44DD549E6E422?d-5470-p=4&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=DEZEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>0</v>
+      </c>
+      <c r="E431" t="n">
+        <v>6</v>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:54:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=5EFB7D6BF60A98EEE9F115E1D24D73B1?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=DEZEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D432" t="n">
+        <v>0</v>
+      </c>
+      <c r="E432" t="n">
+        <v>6</v>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>2026-07-31 23:54:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=B1A5861BC5B9CE4C2AC5091151826F8E?d-5470-p=3&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=DEZEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>0</v>
+      </c>
+      <c r="E433" t="n">
+        <v>6</v>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:00:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CEBFE38EB8AAFA7E61C60AA13BB144FC?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=DEZEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D434" t="n">
+        <v>0</v>
+      </c>
+      <c r="E434" t="n">
+        <v>6</v>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:01:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=BA60F01DB9DBCA80DC4BAF2B3EDA2A18?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=DEZEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D435" t="n">
+        <v>0</v>
+      </c>
+      <c r="E435" t="n">
+        <v>6</v>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:02:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E98D9136531BE17BE2011A91112CBDC9?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2020&amp;d-5470-e=9&amp;formulario.mes=DEZEMBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D436" t="n">
+        <v>0</v>
+      </c>
+      <c r="E436" t="n">
+        <v>6</v>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:05:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=23B51764A9B17D808E223CE425118D56?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=JANEIRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D437" t="n">
+        <v>0</v>
+      </c>
+      <c r="E437" t="n">
+        <v>6</v>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:10:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=7616D65F64398860BCB4AB2FB0905D2E?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=JANEIRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D438" t="n">
+        <v>0</v>
+      </c>
+      <c r="E438" t="n">
+        <v>6</v>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:14:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=2D8451D91E6CA50CE43B59F0C8B6CE93?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=MARCO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D439" t="n">
+        <v>0</v>
+      </c>
+      <c r="E439" t="n">
+        <v>6</v>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:35:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=0C58E2E330E3B747394F6FD884C8171F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=MARCO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D440" t="n">
+        <v>0</v>
+      </c>
+      <c r="E440" t="n">
+        <v>6</v>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:39:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=8B91EC1B046070D6C3DA1DC26C5D547C?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=MARCO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D441" t="n">
+        <v>0</v>
+      </c>
+      <c r="E441" t="n">
+        <v>6</v>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>2026-08-01 00:44:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=5BEC913BCBF509C7B9A040EE6C6F3DD7?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=MAIO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D442" t="n">
+        <v>0</v>
+      </c>
+      <c r="E442" t="n">
+        <v>6</v>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>2026-08-01 01:06:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=20FEB724BE11931BB119C96D158502AE?d-5470-p=3&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=MAIO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D443" t="n">
+        <v>0</v>
+      </c>
+      <c r="E443" t="n">
+        <v>6</v>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>2026-08-01 01:17:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=7A3A6C91150B94CED6924267C3448436?d-5470-p=4&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=JUNHO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D444" t="n">
+        <v>0</v>
+      </c>
+      <c r="E444" t="n">
+        <v>6</v>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>2026-08-01 01:23:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=778500C98514E3A75A9431A66EC9B34F?d-5470-p=3&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=JULHO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D445" t="n">
+        <v>0</v>
+      </c>
+      <c r="E445" t="n">
+        <v>6</v>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>2026-08-01 01:33:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E6E7B396A9C6830DD6F1806C93D51629?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=JULHO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D446" t="n">
+        <v>0</v>
+      </c>
+      <c r="E446" t="n">
+        <v>6</v>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>2026-08-01 01:36:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=216F0B6504C010322EDAD195304D9F0F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=JULHO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D447" t="n">
+        <v>0</v>
+      </c>
+      <c r="E447" t="n">
+        <v>6</v>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>2026-08-01 01:39:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=A6281B5E63B4C32D032C7F8B68DA9D14?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=AGOSTO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D448" t="n">
+        <v>0</v>
+      </c>
+      <c r="E448" t="n">
+        <v>6</v>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>2026-08-01 01:56:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=56494504DC7D61CC7B1F77BE24BFDA9D?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=AGOSTO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D449" t="n">
+        <v>0</v>
+      </c>
+      <c r="E449" t="n">
+        <v>6</v>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>2026-08-01 01:57:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=0D1AA412DE062F7FB61F2894EBA7765B?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D450" t="n">
+        <v>0</v>
+      </c>
+      <c r="E450" t="n">
+        <v>6</v>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>2026-08-01 02:24:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=6A5B5DF6686147B93D7869EC8DFBA619?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2019&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>SELENIUM_ERRO: WebDriverException</t>
+        </is>
+      </c>
+      <c r="D451" t="n">
+        <v>0</v>
+      </c>
+      <c r="E451" t="n">
+        <v>6</v>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>2026-08-01 02:26:15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Resultados PR (Etapa 1)
</commit_message>
<xml_diff>
--- a/resultados/abatia/erros_varredura.xlsx
+++ b/resultados/abatia/erros_varredura.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F733"/>
+  <dimension ref="A1:F774"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20944,6 +20944,1154 @@
         </is>
       </c>
     </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E7BDAA73F83352A0AF37B7DBFA299E9F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=2&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D734" t="n">
+        <v>502</v>
+      </c>
+      <c r="E734" t="n">
+        <v>7</v>
+      </c>
+      <c r="F734" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:47:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E7BDAA73F83352A0AF37B7DBFA299E9F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=5&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D735" t="n">
+        <v>502</v>
+      </c>
+      <c r="E735" t="n">
+        <v>7</v>
+      </c>
+      <c r="F735" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:48:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E7BDAA73F83352A0AF37B7DBFA299E9F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=6&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D736" t="n">
+        <v>502</v>
+      </c>
+      <c r="E736" t="n">
+        <v>7</v>
+      </c>
+      <c r="F736" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:48:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E7BDAA73F83352A0AF37B7DBFA299E9F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=7&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D737" t="n">
+        <v>502</v>
+      </c>
+      <c r="E737" t="n">
+        <v>7</v>
+      </c>
+      <c r="F737" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:48:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E7BDAA73F83352A0AF37B7DBFA299E9F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=8&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D738" t="n">
+        <v>502</v>
+      </c>
+      <c r="E738" t="n">
+        <v>7</v>
+      </c>
+      <c r="F738" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:49:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E7BDAA73F83352A0AF37B7DBFA299E9F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D739" t="n">
+        <v>502</v>
+      </c>
+      <c r="E739" t="n">
+        <v>7</v>
+      </c>
+      <c r="F739" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:49:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E7BDAA73F83352A0AF37B7DBFA299E9F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=10&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D740" t="n">
+        <v>502</v>
+      </c>
+      <c r="E740" t="n">
+        <v>7</v>
+      </c>
+      <c r="F740" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:49:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E7BDAA73F83352A0AF37B7DBFA299E9F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=11&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D741" t="n">
+        <v>502</v>
+      </c>
+      <c r="E741" t="n">
+        <v>7</v>
+      </c>
+      <c r="F741" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:50:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E7BDAA73F83352A0AF37B7DBFA299E9F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=12&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D742" t="n">
+        <v>502</v>
+      </c>
+      <c r="E742" t="n">
+        <v>7</v>
+      </c>
+      <c r="F742" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:51:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E7BDAA73F83352A0AF37B7DBFA299E9F?d-5470-p=1&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=13&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D743" t="n">
+        <v>502</v>
+      </c>
+      <c r="E743" t="n">
+        <v>7</v>
+      </c>
+      <c r="F743" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:51:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=1&amp;formulario.exercicio=2025&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D744" t="n">
+        <v>502</v>
+      </c>
+      <c r="E744" t="n">
+        <v>7</v>
+      </c>
+      <c r="F744" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:51:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=4&amp;formulario.exercicio=2025&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D745" t="n">
+        <v>502</v>
+      </c>
+      <c r="E745" t="n">
+        <v>7</v>
+      </c>
+      <c r="F745" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:52:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=2&amp;formulario.exercicio=2025&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D746" t="n">
+        <v>502</v>
+      </c>
+      <c r="E746" t="n">
+        <v>7</v>
+      </c>
+      <c r="F746" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:52:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=3&amp;formulario.exercicio=2025&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D747" t="n">
+        <v>502</v>
+      </c>
+      <c r="E747" t="n">
+        <v>7</v>
+      </c>
+      <c r="F747" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:52:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=6&amp;formulario.exercicio=2025&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D748" t="n">
+        <v>502</v>
+      </c>
+      <c r="E748" t="n">
+        <v>7</v>
+      </c>
+      <c r="F748" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:53:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=1&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D749" t="n">
+        <v>502</v>
+      </c>
+      <c r="E749" t="n">
+        <v>7</v>
+      </c>
+      <c r="F749" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:53:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=2&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D750" t="n">
+        <v>502</v>
+      </c>
+      <c r="E750" t="n">
+        <v>7</v>
+      </c>
+      <c r="F750" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:54:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=5&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D751" t="n">
+        <v>502</v>
+      </c>
+      <c r="E751" t="n">
+        <v>7</v>
+      </c>
+      <c r="F751" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:54:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=6&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D752" t="n">
+        <v>502</v>
+      </c>
+      <c r="E752" t="n">
+        <v>7</v>
+      </c>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:54:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=7&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D753" t="n">
+        <v>502</v>
+      </c>
+      <c r="E753" t="n">
+        <v>7</v>
+      </c>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:55:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=8&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D754" t="n">
+        <v>502</v>
+      </c>
+      <c r="E754" t="n">
+        <v>7</v>
+      </c>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:55:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D755" t="n">
+        <v>502</v>
+      </c>
+      <c r="E755" t="n">
+        <v>7</v>
+      </c>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:56:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=10&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D756" t="n">
+        <v>502</v>
+      </c>
+      <c r="E756" t="n">
+        <v>7</v>
+      </c>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:56:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=11&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D757" t="n">
+        <v>502</v>
+      </c>
+      <c r="E757" t="n">
+        <v>7</v>
+      </c>
+      <c r="F757" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:57:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=12&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D758" t="n">
+        <v>502</v>
+      </c>
+      <c r="E758" t="n">
+        <v>7</v>
+      </c>
+      <c r="F758" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:57:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=E797095F6C4C2B6E6E52781044B58566?d-5470-p=5&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=13&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D759" t="n">
+        <v>502</v>
+      </c>
+      <c r="E759" t="n">
+        <v>7</v>
+      </c>
+      <c r="F759" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:57:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=1&amp;formulario.exercicio=2025&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D760" t="n">
+        <v>502</v>
+      </c>
+      <c r="E760" t="n">
+        <v>7</v>
+      </c>
+      <c r="F760" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:58:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=3&amp;formulario.exercicio=2025&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D761" t="n">
+        <v>502</v>
+      </c>
+      <c r="E761" t="n">
+        <v>7</v>
+      </c>
+      <c r="F761" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:58:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=4&amp;formulario.exercicio=2025&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D762" t="n">
+        <v>502</v>
+      </c>
+      <c r="E762" t="n">
+        <v>7</v>
+      </c>
+      <c r="F762" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:58:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=5&amp;formulario.exercicio=2025&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D763" t="n">
+        <v>502</v>
+      </c>
+      <c r="E763" t="n">
+        <v>7</v>
+      </c>
+      <c r="F763" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:59:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=6&amp;formulario.exercicio=2025&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D764" t="n">
+        <v>502</v>
+      </c>
+      <c r="E764" t="n">
+        <v>7</v>
+      </c>
+      <c r="F764" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:59:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=1&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D765" t="n">
+        <v>502</v>
+      </c>
+      <c r="E765" t="n">
+        <v>7</v>
+      </c>
+      <c r="F765" t="inlineStr">
+        <is>
+          <t>2026-08-04 06:59:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=2&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D766" t="n">
+        <v>502</v>
+      </c>
+      <c r="E766" t="n">
+        <v>7</v>
+      </c>
+      <c r="F766" t="inlineStr">
+        <is>
+          <t>2026-08-04 07:00:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=5&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D767" t="n">
+        <v>502</v>
+      </c>
+      <c r="E767" t="n">
+        <v>7</v>
+      </c>
+      <c r="F767" t="inlineStr">
+        <is>
+          <t>2026-08-04 07:00:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=6&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D768" t="n">
+        <v>502</v>
+      </c>
+      <c r="E768" t="n">
+        <v>7</v>
+      </c>
+      <c r="F768" t="inlineStr">
+        <is>
+          <t>2026-08-04 07:01:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=7&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D769" t="n">
+        <v>502</v>
+      </c>
+      <c r="E769" t="n">
+        <v>7</v>
+      </c>
+      <c r="F769" t="inlineStr">
+        <is>
+          <t>2026-08-04 07:01:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=8&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D770" t="n">
+        <v>502</v>
+      </c>
+      <c r="E770" t="n">
+        <v>7</v>
+      </c>
+      <c r="F770" t="inlineStr">
+        <is>
+          <t>2026-08-04 07:02:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=9&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D771" t="n">
+        <v>502</v>
+      </c>
+      <c r="E771" t="n">
+        <v>7</v>
+      </c>
+      <c r="F771" t="inlineStr">
+        <is>
+          <t>2026-08-04 07:02:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=10&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>HTTP_502</t>
+        </is>
+      </c>
+      <c r="D772" t="n">
+        <v>502</v>
+      </c>
+      <c r="E772" t="n">
+        <v>7</v>
+      </c>
+      <c r="F772" t="inlineStr">
+        <is>
+          <t>2026-08-04 07:03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=11&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>TIMEOUT_OU_CONEXAO</t>
+        </is>
+      </c>
+      <c r="D773" t="n">
+        <v>0</v>
+      </c>
+      <c r="E773" t="n">
+        <v>7</v>
+      </c>
+      <c r="F773" t="inlineStr">
+        <is>
+          <t>2026-08-04 07:05:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>abatia</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>https://abatia.metajuris.com.br/transparencia/srhRelacaoDeServidoresAtivos/listData;jsessionid=CA1BCD19B361EB72DD954D322A3344BD?d-5470-p=2&amp;6578706f7274=1&amp;formulario.exercicio=2025&amp;d-5470-e=12&amp;formulario.mes=OUTUBRO&amp;formulario.codEntidade=249</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>TIMEOUT_OU_CONEXAO</t>
+        </is>
+      </c>
+      <c r="D774" t="n">
+        <v>0</v>
+      </c>
+      <c r="E774" t="n">
+        <v>7</v>
+      </c>
+      <c r="F774" t="inlineStr">
+        <is>
+          <t>2026-08-04 07:07:46</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>